<commit_message>
ECS-93 added hyperlinks in evaluation-results-history xlsx report
</commit_message>
<xml_diff>
--- a/eca-ers/src/main/resources/report-templates/evaluation-results-history-report-template.xlsx
+++ b/eca-ers/src/main/resources/report-templates/evaluation-results-history-report-template.xlsx
@@ -12,7 +12,6 @@
     <sheet name="Лист3" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="124519"/>
-  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
@@ -286,16 +285,6 @@
     </r>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-      </rPr>
-      <t>${item.classifierName}</t>
-    </r>
-  </si>
-  <si>
     <t>${item.relationName}</t>
   </si>
   <si>
@@ -352,6 +341,9 @@
   </si>
   <si>
     <t>Страница ${report.page} из ${report.totalPages}</t>
+  </si>
+  <si>
+    <t>${util.hyperlink(item.requestPathUrl, item.classifierName)}</t>
   </si>
 </sst>
 </file>
@@ -377,11 +369,6 @@
       <name val="Calibri"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
       <sz val="9"/>
       <color indexed="81"/>
       <name val="Tahoma"/>
@@ -393,6 +380,14 @@
       <color indexed="81"/>
       <name val="Tahoma"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
     </font>
   </fonts>
   <fills count="6">
@@ -504,23 +499,23 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -758,18 +753,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="15.6">
-      <c r="A1" s="11" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="11"/>
-      <c r="C1" s="11"/>
-      <c r="D1" s="11"/>
-      <c r="E1" s="11"/>
-      <c r="F1" s="11"/>
-      <c r="G1" s="11"/>
-      <c r="H1" s="11"/>
-      <c r="I1" s="11"/>
-      <c r="J1" s="11"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13"/>
+      <c r="I1" s="13"/>
+      <c r="J1" s="13"/>
     </row>
     <row r="2" spans="1:15" ht="15.6">
       <c r="A2" s="1"/>
@@ -787,65 +782,65 @@
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="12" t="s">
+      <c r="B3" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="12"/>
-      <c r="D3" s="12"/>
-      <c r="E3" s="12"/>
-      <c r="F3" s="12"/>
-      <c r="G3" s="12"/>
-      <c r="H3" s="12"/>
-      <c r="I3" s="12"/>
-      <c r="J3" s="12"/>
+      <c r="C3" s="14"/>
+      <c r="D3" s="14"/>
+      <c r="E3" s="14"/>
+      <c r="F3" s="14"/>
+      <c r="G3" s="14"/>
+      <c r="H3" s="14"/>
+      <c r="I3" s="14"/>
+      <c r="J3" s="14"/>
     </row>
     <row r="4" spans="1:15" ht="14.85" customHeight="1">
       <c r="A4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="13" t="s">
+      <c r="B4" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="13"/>
-      <c r="D4" s="13"/>
-      <c r="E4" s="13"/>
-      <c r="F4" s="13"/>
-      <c r="G4" s="13"/>
-      <c r="H4" s="13"/>
-      <c r="I4" s="13"/>
-      <c r="J4" s="13"/>
+      <c r="C4" s="15"/>
+      <c r="D4" s="15"/>
+      <c r="E4" s="15"/>
+      <c r="F4" s="15"/>
+      <c r="G4" s="15"/>
+      <c r="H4" s="15"/>
+      <c r="I4" s="15"/>
+      <c r="J4" s="15"/>
     </row>
     <row r="5" spans="1:15" ht="14.85" customHeight="1">
       <c r="A5" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="13" t="s">
+      <c r="B5" s="15" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="13"/>
-      <c r="D5" s="13"/>
-      <c r="E5" s="13"/>
-      <c r="F5" s="13"/>
-      <c r="G5" s="13"/>
-      <c r="H5" s="13"/>
-      <c r="I5" s="13"/>
-      <c r="J5" s="13"/>
+      <c r="C5" s="15"/>
+      <c r="D5" s="15"/>
+      <c r="E5" s="15"/>
+      <c r="F5" s="15"/>
+      <c r="G5" s="15"/>
+      <c r="H5" s="15"/>
+      <c r="I5" s="15"/>
+      <c r="J5" s="15"/>
     </row>
     <row r="6" spans="1:15" ht="14.85" customHeight="1">
       <c r="A6" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="13" t="s">
+      <c r="B6" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="13"/>
-      <c r="D6" s="13"/>
-      <c r="E6" s="13"/>
-      <c r="F6" s="13"/>
-      <c r="G6" s="13"/>
-      <c r="H6" s="13"/>
-      <c r="I6" s="13"/>
-      <c r="J6" s="13"/>
+      <c r="C6" s="15"/>
+      <c r="D6" s="15"/>
+      <c r="E6" s="15"/>
+      <c r="F6" s="15"/>
+      <c r="G6" s="15"/>
+      <c r="H6" s="15"/>
+      <c r="I6" s="15"/>
+      <c r="J6" s="15"/>
     </row>
     <row r="7" spans="1:15">
       <c r="A7" s="2"/>
@@ -897,50 +892,50 @@
       <c r="O8" s="7"/>
     </row>
     <row r="9" spans="1:15" ht="15" customHeight="1">
-      <c r="A9" s="8" t="s">
+      <c r="A9" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="B9" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="B9" s="9" t="s">
+      <c r="C9" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="C9" s="9" t="s">
+      <c r="D9" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="D9" s="9" t="s">
+      <c r="E9" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="E9" s="9" t="s">
+      <c r="F9" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="F9" s="9" t="s">
+      <c r="G9" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="G9" s="9" t="s">
+      <c r="H9" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="H9" s="9" t="s">
+      <c r="I9" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="I9" s="10" t="s">
+      <c r="J9" s="8" t="s">
         <v>25</v>
-      </c>
-      <c r="J9" s="9" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="10" spans="1:15">
-      <c r="A10" s="14" t="s">
-        <v>27</v>
-      </c>
-      <c r="B10" s="15"/>
-      <c r="C10" s="15"/>
-      <c r="D10" s="15"/>
-      <c r="E10" s="15"/>
-      <c r="F10" s="15"/>
-      <c r="G10" s="15"/>
-      <c r="H10" s="15"/>
-      <c r="I10" s="15"/>
-      <c r="J10" s="16"/>
+      <c r="A10" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="B10" s="11"/>
+      <c r="C10" s="11"/>
+      <c r="D10" s="11"/>
+      <c r="E10" s="11"/>
+      <c r="F10" s="11"/>
+      <c r="G10" s="11"/>
+      <c r="H10" s="11"/>
+      <c r="I10" s="11"/>
+      <c r="J10" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -952,8 +947,8 @@
     <mergeCell ref="B6:J6"/>
   </mergeCells>
   <pageMargins left="0.70000004768371604" right="0.70000004768371604" top="0.75" bottom="0.75" header="0.51180553436279297" footer="0.51180553436279297"/>
-  <pageSetup paperSize="9" fitToWidth="0" fitToHeight="0" orientation="portrait"/>
-  <legacyDrawing r:id="rId1"/>
+  <pageSetup paperSize="9" fitToWidth="0" fitToHeight="0" orientation="portrait" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
ECS-98 added extended classifiers options in evaluation-results-history-report-template.xlsx
</commit_message>
<xml_diff>
--- a/eca-ers/src/main/resources/report-templates/evaluation-results-history-report-template.xlsx
+++ b/eca-ers/src/main/resources/report-templates/evaluation-results-history-report-template.xlsx
@@ -482,7 +482,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
@@ -505,6 +505,12 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -513,9 +519,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -753,18 +756,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="15.6">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
-      <c r="H1" s="13"/>
-      <c r="I1" s="13"/>
-      <c r="J1" s="13"/>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
+      <c r="H1" s="15"/>
+      <c r="I1" s="15"/>
+      <c r="J1" s="15"/>
     </row>
     <row r="2" spans="1:15" ht="15.6">
       <c r="A2" s="1"/>
@@ -782,65 +785,65 @@
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="14" t="s">
+      <c r="B3" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="14"/>
-      <c r="D3" s="14"/>
-      <c r="E3" s="14"/>
-      <c r="F3" s="14"/>
-      <c r="G3" s="14"/>
-      <c r="H3" s="14"/>
-      <c r="I3" s="14"/>
-      <c r="J3" s="14"/>
+      <c r="C3" s="16"/>
+      <c r="D3" s="16"/>
+      <c r="E3" s="16"/>
+      <c r="F3" s="16"/>
+      <c r="G3" s="16"/>
+      <c r="H3" s="16"/>
+      <c r="I3" s="16"/>
+      <c r="J3" s="16"/>
     </row>
     <row r="4" spans="1:15" ht="14.85" customHeight="1">
       <c r="A4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="15" t="s">
+      <c r="B4" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="15"/>
-      <c r="D4" s="15"/>
-      <c r="E4" s="15"/>
-      <c r="F4" s="15"/>
-      <c r="G4" s="15"/>
-      <c r="H4" s="15"/>
-      <c r="I4" s="15"/>
-      <c r="J4" s="15"/>
+      <c r="C4" s="17"/>
+      <c r="D4" s="17"/>
+      <c r="E4" s="17"/>
+      <c r="F4" s="17"/>
+      <c r="G4" s="17"/>
+      <c r="H4" s="17"/>
+      <c r="I4" s="17"/>
+      <c r="J4" s="17"/>
     </row>
     <row r="5" spans="1:15" ht="14.85" customHeight="1">
       <c r="A5" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="15" t="s">
+      <c r="B5" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="15"/>
-      <c r="D5" s="15"/>
-      <c r="E5" s="15"/>
-      <c r="F5" s="15"/>
-      <c r="G5" s="15"/>
-      <c r="H5" s="15"/>
-      <c r="I5" s="15"/>
-      <c r="J5" s="15"/>
+      <c r="C5" s="17"/>
+      <c r="D5" s="17"/>
+      <c r="E5" s="17"/>
+      <c r="F5" s="17"/>
+      <c r="G5" s="17"/>
+      <c r="H5" s="17"/>
+      <c r="I5" s="17"/>
+      <c r="J5" s="17"/>
     </row>
     <row r="6" spans="1:15" ht="14.85" customHeight="1">
       <c r="A6" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="15" t="s">
+      <c r="B6" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="15"/>
-      <c r="D6" s="15"/>
-      <c r="E6" s="15"/>
-      <c r="F6" s="15"/>
-      <c r="G6" s="15"/>
-      <c r="H6" s="15"/>
-      <c r="I6" s="15"/>
-      <c r="J6" s="15"/>
+      <c r="C6" s="17"/>
+      <c r="D6" s="17"/>
+      <c r="E6" s="17"/>
+      <c r="F6" s="17"/>
+      <c r="G6" s="17"/>
+      <c r="H6" s="17"/>
+      <c r="I6" s="17"/>
+      <c r="J6" s="17"/>
     </row>
     <row r="7" spans="1:15">
       <c r="A7" s="2"/>
@@ -892,7 +895,7 @@
       <c r="O8" s="7"/>
     </row>
     <row r="9" spans="1:15" ht="15" customHeight="1">
-      <c r="A9" s="16" t="s">
+      <c r="A9" s="10" t="s">
         <v>27</v>
       </c>
       <c r="B9" s="8" t="s">
@@ -901,7 +904,7 @@
       <c r="C9" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="D9" s="8" t="s">
+      <c r="D9" s="11" t="s">
         <v>19</v>
       </c>
       <c r="E9" s="8" t="s">
@@ -924,18 +927,18 @@
       </c>
     </row>
     <row r="10" spans="1:15">
-      <c r="A10" s="10" t="s">
+      <c r="A10" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="B10" s="11"/>
-      <c r="C10" s="11"/>
-      <c r="D10" s="11"/>
-      <c r="E10" s="11"/>
-      <c r="F10" s="11"/>
-      <c r="G10" s="11"/>
-      <c r="H10" s="11"/>
-      <c r="I10" s="11"/>
-      <c r="J10" s="12"/>
+      <c r="B10" s="13"/>
+      <c r="C10" s="13"/>
+      <c r="D10" s="13"/>
+      <c r="E10" s="13"/>
+      <c r="F10" s="13"/>
+      <c r="G10" s="13"/>
+      <c r="H10" s="13"/>
+      <c r="I10" s="13"/>
+      <c r="J10" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="6">

</xml_diff>

<commit_message>
ECS-98 added extended instances info in evaluation-results-history-report-template.xlsx
</commit_message>
<xml_diff>
--- a/eca-ers/src/main/resources/report-templates/evaluation-results-history-report-template.xlsx
+++ b/eca-ers/src/main/resources/report-templates/evaluation-results-history-report-template.xlsx
@@ -285,9 +285,6 @@
     </r>
   </si>
   <si>
-    <t>${item.relationName}</t>
-  </si>
-  <si>
     <t>${item.evaluationMethod}</t>
   </si>
   <si>
@@ -344,13 +341,20 @@
   </si>
   <si>
     <t>${util.hyperlink(item.requestPathUrl, item.classifierName)}</t>
+  </si>
+  <si>
+    <t>${item.relationName}
+Число объектов: ${item.numInstances}
+Число атрибутов: ${item.numAttributes}
+Число классов: ${item.numClasses}
+Атрибут класса: ${item.className}</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -385,6 +389,13 @@
       <b/>
       <sz val="11"/>
       <color theme="3"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="204"/>
@@ -482,7 +493,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
@@ -519,6 +530,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -896,39 +910,39 @@
     </row>
     <row r="9" spans="1:15" ht="15" customHeight="1">
       <c r="A9" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="B9" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="B9" s="8" t="s">
+      <c r="C9" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="C9" s="8" t="s">
+      <c r="D9" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="D9" s="11" t="s">
+      <c r="E9" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="E9" s="8" t="s">
+      <c r="F9" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="F9" s="8" t="s">
+      <c r="G9" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="G9" s="8" t="s">
+      <c r="H9" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="H9" s="8" t="s">
+      <c r="I9" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="I9" s="9" t="s">
+      <c r="J9" s="8" t="s">
         <v>24</v>
-      </c>
-      <c r="J9" s="8" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="10" spans="1:15">
       <c r="A10" s="12" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B10" s="13"/>
       <c r="C10" s="13"/>

</xml_diff>